<commit_message>
added required steps for installation - for linux
</commit_message>
<xml_diff>
--- a/dementia_features_log.xlsx
+++ b/dementia_features_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -834,7 +834,57 @@
       <c r="N7" t="n">
         <v>0.535872</v>
       </c>
-      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-21 17:42:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>microphone</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>No Dementia</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="E8" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>40.75</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.473852</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-2.424608</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8.239912</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.052976</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.041608</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="M8" t="n">
+        <v>13.977428</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.103986</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>